<commit_message>
Tu mensaje de cambio
</commit_message>
<xml_diff>
--- a/Modelo OEE.xlsx
+++ b/Modelo OEE.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr hidePivotFieldList="1"/>
   <bookViews>
-    <workbookView windowWidth="18431" windowHeight="6451"/>
+    <workbookView windowWidth="17591" windowHeight="6451"/>
   </bookViews>
   <sheets>
     <sheet name="Por hora" sheetId="2" r:id="rId1"/>
@@ -290,7 +290,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="70">
+  <si>
+    <t>OEE esperado</t>
+  </si>
   <si>
     <t>Producción Planeada</t>
   </si>
@@ -353,6 +356,9 @@
   </si>
   <si>
     <t>%</t>
+  </si>
+  <si>
+    <t>OEE esperado*VN*TP</t>
   </si>
   <si>
     <t>Dato</t>
@@ -511,7 +517,7 @@
     <numFmt numFmtId="181" formatCode="0.0000"/>
     <numFmt numFmtId="182" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="30">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -534,12 +540,24 @@
     </font>
     <font>
       <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color rgb="FF0432FF"/>
+      <name val="Times New Roman"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <name val="Times New Roman"/>
       <charset val="134"/>
     </font>
     <font>
       <sz val="12"/>
+      <color rgb="FF0432FF"/>
       <name val="Times New Roman"/>
       <charset val="134"/>
     </font>
@@ -704,17 +722,17 @@
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
-      <name val="Tahoma"/>
+      <name val="Aptos Narrow"/>
       <charset val="134"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
+      <name val="Tahoma"/>
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -725,6 +743,12 @@
       <patternFill patternType="solid">
         <fgColor theme="2"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE8E8E8"/>
+        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
     <fill>
@@ -938,9 +962,26 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
-      <right/>
-      <top/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
@@ -962,22 +1003,7 @@
     <border>
       <left/>
       <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
+      <top/>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
@@ -985,13 +1011,11 @@
     </border>
     <border>
       <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
+      <right/>
       <top style="thin">
         <color auto="1"/>
       </top>
-      <bottom style="thin">
+      <bottom style="medium">
         <color auto="1"/>
       </bottom>
       <diagonal/>
@@ -1097,24 +1121,15 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="42" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1123,122 +1138,131 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="7" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="5" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1248,80 +1272,89 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="16" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="20" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="0" xfId="4" applyFont="1" applyFill="1"/>
-    <xf numFmtId="177" fontId="4" fillId="0" borderId="0" xfId="4" applyFont="1" applyFill="1"/>
-    <xf numFmtId="177" fontId="4" fillId="0" borderId="4" xfId="4" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="177" fontId="6" fillId="0" borderId="0" xfId="4" applyFont="1" applyFill="1"/>
     <xf numFmtId="177" fontId="1" fillId="0" borderId="0" xfId="4" applyFont="1" applyFill="1"/>
-    <xf numFmtId="178" fontId="3" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="179" fontId="3" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="178" fontId="6" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="179" fontId="6" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="179" fontId="1" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="180" fontId="3" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="180" fontId="6" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="177" fontId="5" fillId="0" borderId="0" xfId="4" applyFont="1" applyFill="1"/>
     <xf numFmtId="181" fontId="1" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="178" fontId="4" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="179" fontId="4" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="181" fontId="4" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="178" fontId="4" fillId="0" borderId="4" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="179" fontId="4" fillId="0" borderId="4" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="181" fontId="4" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="10" fontId="1" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="10" fontId="4" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+    <xf numFmtId="178" fontId="5" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="179" fontId="5" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="181" fontId="5" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="5" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="10" fontId="4" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="4" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="5" fillId="0" borderId="6" xfId="4" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="178" fontId="5" fillId="0" borderId="6" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="179" fontId="5" fillId="0" borderId="6" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="181" fontId="5" fillId="0" borderId="6" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="5" fillId="0" borderId="6" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="6" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="182" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Coma" xfId="1" builtinId="3"/>
     <cellStyle name="Moneda" xfId="2" builtinId="4"/>
-    <cellStyle name="Porcentaje" xfId="3" builtinId="5"/>
+    <cellStyle name="K" xfId="3" builtinId="5"/>
     <cellStyle name="Coma [0]" xfId="4" builtinId="6"/>
     <cellStyle name="Moneda [0]" xfId="5" builtinId="7"/>
     <cellStyle name="Hipervínculo" xfId="6" builtinId="8"/>
@@ -2015,7 +2048,10 @@
     <col min="2" max="2" width="15.1231884057971" customWidth="1"/>
     <col min="3" max="3" width="11.6231884057971" customWidth="1"/>
     <col min="4" max="4" width="12.6231884057971" customWidth="1"/>
-    <col min="5" max="8" width="10.6231884057971" customWidth="1"/>
+    <col min="5" max="5" width="8.93478260869565" customWidth="1"/>
+    <col min="6" max="6" width="7.84057971014493" customWidth="1"/>
+    <col min="7" max="7" width="13.9420289855072" customWidth="1"/>
+    <col min="8" max="8" width="10.6231884057971" customWidth="1"/>
     <col min="9" max="9" width="11.8768115942029" customWidth="1"/>
     <col min="10" max="10" width="10.3768115942029" customWidth="1"/>
     <col min="11" max="12" width="10.1231884057971" customWidth="1"/>
@@ -2032,878 +2068,891 @@
     <col min="23" max="23" width="5.8768115942029" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="7:22">
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
-      <c r="I1" s="5"/>
-      <c r="J1" s="5"/>
-      <c r="K1" s="5"/>
-      <c r="L1" s="5"/>
-      <c r="M1" s="5"/>
-      <c r="N1" s="5"/>
-      <c r="O1" s="5"/>
-      <c r="P1" s="16"/>
-      <c r="Q1" s="16"/>
-      <c r="R1" s="5"/>
-      <c r="S1" s="5"/>
-      <c r="T1" s="5"/>
-      <c r="U1" s="5"/>
-      <c r="V1" s="5"/>
+    <row r="1" s="1" customFormat="1" spans="1:22">
+      <c r="G1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="6"/>
+      <c r="L1" s="6"/>
+      <c r="M1" s="6"/>
+      <c r="N1" s="6"/>
+      <c r="O1" s="6"/>
+      <c r="P1" s="7"/>
+      <c r="Q1" s="7"/>
+      <c r="R1" s="6"/>
+      <c r="S1" s="6"/>
+      <c r="T1" s="6"/>
+      <c r="U1" s="6"/>
+      <c r="V1" s="6"/>
     </row>
-    <row r="2" s="1" customFormat="1" spans="3:17">
-      <c r="C2" s="6"/>
-      <c r="P2" s="17"/>
-      <c r="Q2" s="17"/>
+    <row r="2" s="1" customFormat="1" spans="1:22">
+      <c r="C2" s="8"/>
+      <c r="G2" s="9">
+        <v>0.7</v>
+      </c>
+      <c r="P2" s="10"/>
+      <c r="Q2" s="10"/>
     </row>
-    <row r="3" s="2" customFormat="1" ht="46.65" spans="7:22">
-      <c r="G3" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="H3" s="7" t="s">
+    <row r="3" s="2" customFormat="1" ht="46.65" spans="1:22">
+      <c r="G3" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="I3" s="7" t="s">
+      <c r="H3" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="J3" s="7" t="s">
+      <c r="I3" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="K3" s="7" t="s">
+      <c r="J3" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="L3" s="7" t="s">
+      <c r="K3" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="M3" s="7" t="s">
+      <c r="L3" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="N3" s="7" t="s">
+      <c r="M3" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="O3" s="18" t="s">
+      <c r="N3" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="P3" s="7" t="s">
+      <c r="O3" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="Q3" s="7" t="s">
+      <c r="P3" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="R3" s="35" t="s">
+      <c r="Q3" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="S3" s="7" t="s">
+      <c r="R3" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="T3" s="7" t="s">
+      <c r="S3" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="U3" s="7" t="s">
+      <c r="T3" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="V3" s="7" t="s">
+      <c r="U3" s="11" t="s">
         <v>15</v>
       </c>
+      <c r="V3" s="11" t="s">
+        <v>16</v>
+      </c>
     </row>
-    <row r="4" s="2" customFormat="1" spans="7:22">
-      <c r="G4" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="H4" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="I4" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="J4" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="K4" s="8" t="s">
+    <row r="4" s="2" customFormat="1" spans="1:22">
+      <c r="G4" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="L4" s="8" t="s">
+      <c r="H4" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="M4" s="8" t="s">
+      <c r="I4" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="N4" s="19" t="s">
+      <c r="J4" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="K4" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="O4" s="8" t="s">
+      <c r="L4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="M4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="N4" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="P4" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="Q4" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="R4" s="7" t="s">
+      <c r="O4" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="S4" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="T4" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="U4" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="V4" s="8" t="s">
-        <v>20</v>
+      <c r="P4" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q4" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="R4" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="S4" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="T4" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="U4" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="V4" s="14" t="s">
+        <v>21</v>
       </c>
     </row>
-    <row r="5" s="2" customFormat="1" spans="1:22">
-      <c r="A5" s="9"/>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="I5" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="J5" s="21" t="s">
+    <row r="5" s="2" customFormat="1" ht="31.1" spans="1:22">
+      <c r="A5" s="17"/>
+      <c r="B5" s="17"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="17"/>
+      <c r="G5" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="K5" s="7" t="s">
+      <c r="H5" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="L5" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="M5" s="7" t="s">
+      <c r="I5" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="J5" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="N5" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="O5" s="7" t="s">
+      <c r="K5" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="P5" s="7" t="s">
+      <c r="L5" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="M5" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="Q5" s="7" t="s">
+      <c r="N5" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="O5" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="R5" s="7" t="s">
+      <c r="P5" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="S5" s="7" t="s">
+      <c r="Q5" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="T5" s="7" t="s">
+      <c r="R5" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="U5" s="7" t="s">
+      <c r="S5" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="V5" s="7" t="s">
+      <c r="T5" s="11" t="s">
         <v>32</v>
+      </c>
+      <c r="U5" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="V5" s="11" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="6" s="3" customFormat="1" spans="1:22">
-      <c r="A6" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="C6" s="10" t="s">
+      <c r="A6" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="B6" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="C6" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="D6" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="G6" s="10" t="s">
+      <c r="E6" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="H6" s="10" t="s">
+      <c r="F6" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="I6" s="10" t="s">
+      <c r="G6" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="J6" s="10" t="s">
+      <c r="H6" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="K6" s="10" t="s">
+      <c r="I6" s="20" t="s">
         <v>43</v>
       </c>
-      <c r="L6" s="10" t="s">
+      <c r="J6" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="M6" s="10" t="s">
+      <c r="K6" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="N6" s="10" t="s">
+      <c r="L6" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="O6" s="10" t="s">
+      <c r="M6" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="P6" s="10" t="s">
+      <c r="N6" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="Q6" s="10" t="s">
+      <c r="O6" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="R6" s="10" t="s">
+      <c r="P6" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="S6" s="10" t="s">
+      <c r="Q6" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="T6" s="10" t="s">
+      <c r="R6" s="20" t="s">
         <v>52</v>
       </c>
-      <c r="U6" s="10" t="s">
+      <c r="S6" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="V6" s="10" t="s">
+      <c r="T6" s="20" t="s">
         <v>54</v>
+      </c>
+      <c r="U6" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="V6" s="20" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="7" s="4" customFormat="1" spans="1:22">
-      <c r="A7" s="11">
+      <c r="A7" s="21">
         <v>46078</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="E7" s="12">
+        <v>59</v>
+      </c>
+      <c r="E7" s="22">
         <v>0.25</v>
       </c>
-      <c r="F7" s="12">
+      <c r="F7" s="22">
         <v>0.291666666666667</v>
       </c>
-      <c r="G7" s="13">
-        <v>1840</v>
-      </c>
-      <c r="H7" s="13">
+      <c r="G7" s="23">
+        <f t="shared" ref="G7:G14" si="0">$G$2*O7*K7</f>
+        <v>2459.8</v>
+      </c>
+      <c r="H7" s="23">
         <v>1755</v>
       </c>
-      <c r="I7" s="13">
+      <c r="I7" s="23">
         <v>64</v>
       </c>
-      <c r="J7" s="22">
+      <c r="J7" s="24">
         <v>1691</v>
       </c>
-      <c r="K7" s="23">
+      <c r="K7" s="25">
         <v>1</v>
       </c>
-      <c r="L7" s="24">
+      <c r="L7" s="26">
         <v>0.3</v>
       </c>
-      <c r="M7" s="25">
-        <f t="shared" ref="M7:M19" si="0">K7-L7</f>
+      <c r="M7" s="27">
+        <f t="shared" ref="M7:M19" si="1">K7-L7</f>
         <v>0.7</v>
       </c>
-      <c r="N7" s="26">
+      <c r="N7" s="28">
         <v>0.000284575981787137</v>
       </c>
-      <c r="O7" s="14">
-        <f t="shared" ref="O7:O19" si="1">1/N7</f>
+      <c r="O7" s="29">
+        <f t="shared" ref="O7:O19" si="2">1/N7</f>
         <v>3514</v>
       </c>
-      <c r="P7" s="27">
-        <f>IF(M7=0," ",IFERROR(IF($P$1=1,H7/O7,H7*N7)," "))</f>
+      <c r="P7" s="30">
+        <f t="shared" ref="P7:P19" si="3">IF(M7=0," ",IFERROR(IF($P$1=1,H7/O7,H7*N7)," "))</f>
         <v>0.499430848036425</v>
       </c>
-      <c r="Q7" s="27">
-        <f>IFERROR(IF($Q$1=1,J7/O7,J7*N7)," ")</f>
+      <c r="Q7" s="30">
+        <f t="shared" ref="Q7:Q19" si="4">IFERROR(IF($Q$1=1,J7/O7,J7*N7)," ")</f>
         <v>0.481217985202049</v>
       </c>
-      <c r="R7" s="36">
-        <f t="shared" ref="R7:R20" si="2">IFERROR(M7/K7," ")</f>
+      <c r="R7" s="31">
+        <f t="shared" ref="R7:R20" si="5">IFERROR(M7/K7," ")</f>
         <v>0.7</v>
       </c>
-      <c r="S7" s="36">
-        <f t="shared" ref="S7:S20" si="3">IFERROR(P7/M7," ")</f>
+      <c r="S7" s="31">
+        <f t="shared" ref="S7:S20" si="6">IFERROR(P7/M7," ")</f>
         <v>0.713472640052036</v>
       </c>
-      <c r="T7" s="36">
-        <f t="shared" ref="T7:T20" si="4">IFERROR(Q7/P7," ")</f>
-        <v>0.963532763532765</v>
-      </c>
-      <c r="U7" s="36">
-        <f t="shared" ref="U7:U20" si="5">IFERROR(Q7/K7," ")</f>
+      <c r="T7" s="31">
+        <f t="shared" ref="T7:T20" si="7">IFERROR(Q7/P7," ")</f>
+        <v>0.963532763532764</v>
+      </c>
+      <c r="U7" s="31">
+        <f t="shared" ref="U7:U20" si="8">IFERROR(Q7/K7," ")</f>
         <v>0.481217985202049</v>
       </c>
-      <c r="V7" s="37">
-        <f t="shared" ref="V7:V20" si="6">H7/G7</f>
-        <v>0.953804347826087</v>
+      <c r="V7" s="32">
+        <f t="shared" ref="V7:V20" si="9">H7/G7</f>
+        <v>0.713472640052037</v>
       </c>
     </row>
     <row r="8" s="4" customFormat="1" spans="1:22">
-      <c r="A8" s="11">
+      <c r="A8" s="21">
         <v>46078</v>
       </c>
       <c r="B8" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>56</v>
-      </c>
       <c r="D8" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="E8" s="12">
+        <v>59</v>
+      </c>
+      <c r="E8" s="22">
         <f>F7</f>
         <v>0.291666666666667</v>
       </c>
-      <c r="F8" s="12">
+      <c r="F8" s="22">
         <v>0.333333333333333</v>
       </c>
-      <c r="G8" s="13">
-        <v>1857</v>
-      </c>
-      <c r="H8" s="13">
+      <c r="G8" s="23">
+        <f t="shared" si="0"/>
+        <v>2149</v>
+      </c>
+      <c r="H8" s="23">
         <v>1519</v>
       </c>
-      <c r="I8" s="13">
+      <c r="I8" s="23">
         <v>57</v>
       </c>
-      <c r="J8" s="22">
+      <c r="J8" s="24">
         <v>1462</v>
       </c>
-      <c r="K8" s="23">
+      <c r="K8" s="25">
         <v>1</v>
       </c>
-      <c r="L8" s="24">
+      <c r="L8" s="26">
         <v>0.2</v>
       </c>
-      <c r="M8" s="25">
-        <f t="shared" si="0"/>
+      <c r="M8" s="27">
+        <f t="shared" si="1"/>
         <v>0.8</v>
       </c>
-      <c r="N8" s="26">
+      <c r="N8" s="28">
         <v>0.000325732899022801</v>
       </c>
-      <c r="O8" s="14">
-        <f t="shared" si="1"/>
+      <c r="O8" s="29">
+        <f t="shared" si="2"/>
         <v>3070</v>
       </c>
-      <c r="P8" s="27">
-        <f>IF(M8=0," ",IFERROR(IF($P$1=1,H8/O8,H8*N8)," "))</f>
+      <c r="P8" s="30">
+        <f t="shared" si="3"/>
         <v>0.494788273615635</v>
       </c>
-      <c r="Q8" s="27">
-        <f>IFERROR(IF($Q$1=1,J8/O8,J8*N8)," ")</f>
+      <c r="Q8" s="30">
+        <f t="shared" si="4"/>
         <v>0.476221498371335</v>
       </c>
-      <c r="R8" s="36">
-        <f t="shared" si="2"/>
+      <c r="R8" s="31">
+        <f t="shared" si="5"/>
         <v>0.8</v>
       </c>
-      <c r="S8" s="36">
-        <f t="shared" si="3"/>
-        <v>0.618485342019544</v>
-      </c>
-      <c r="T8" s="36">
-        <f t="shared" si="4"/>
+      <c r="S8" s="31">
+        <f t="shared" si="6"/>
+        <v>0.618485342019543</v>
+      </c>
+      <c r="T8" s="31">
+        <f t="shared" si="7"/>
         <v>0.962475312705727</v>
       </c>
-      <c r="U8" s="36">
-        <f t="shared" si="5"/>
+      <c r="U8" s="31">
+        <f t="shared" si="8"/>
         <v>0.476221498371335</v>
       </c>
-      <c r="V8" s="37">
-        <f t="shared" si="6"/>
-        <v>0.817985998922994</v>
+      <c r="V8" s="32">
+        <f t="shared" si="9"/>
+        <v>0.706840390879479</v>
       </c>
     </row>
     <row r="9" s="4" customFormat="1" spans="1:22">
-      <c r="A9" s="11">
+      <c r="A9" s="21">
         <v>46078</v>
       </c>
       <c r="B9" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="D9" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="C9" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="E9" s="12">
+      <c r="E9" s="22">
         <f>F8</f>
         <v>0.333333333333333</v>
       </c>
-      <c r="F9" s="12">
+      <c r="F9" s="22">
         <v>0.375</v>
       </c>
-      <c r="G9" s="13">
-        <v>1887</v>
-      </c>
-      <c r="H9" s="13">
+      <c r="G9" s="23">
+        <f t="shared" si="0"/>
+        <v>2255.4</v>
+      </c>
+      <c r="H9" s="23">
         <v>1501</v>
       </c>
-      <c r="I9" s="13">
+      <c r="I9" s="23">
         <v>29</v>
       </c>
-      <c r="J9" s="22">
+      <c r="J9" s="24">
         <v>1472</v>
       </c>
-      <c r="K9" s="23">
+      <c r="K9" s="25">
         <v>1</v>
       </c>
-      <c r="L9" s="24">
+      <c r="L9" s="26">
         <v>0.24</v>
       </c>
-      <c r="M9" s="25">
-        <f t="shared" si="0"/>
+      <c r="M9" s="27">
+        <f t="shared" si="1"/>
         <v>0.76</v>
       </c>
-      <c r="N9" s="26">
+      <c r="N9" s="28">
         <v>0.000310366232153942</v>
       </c>
-      <c r="O9" s="14">
-        <f t="shared" si="1"/>
+      <c r="O9" s="29">
+        <f t="shared" si="2"/>
         <v>3222</v>
       </c>
-      <c r="P9" s="27">
-        <f>IF(M9=0," ",IFERROR(IF($P$1=1,H9/O9,H9*N9)," "))</f>
+      <c r="P9" s="30">
+        <f t="shared" si="3"/>
         <v>0.465859714463067</v>
       </c>
-      <c r="Q9" s="27">
-        <f>IFERROR(IF($Q$1=1,J9/O9,J9*N9)," ")</f>
+      <c r="Q9" s="30">
+        <f t="shared" si="4"/>
         <v>0.456859093730603</v>
       </c>
-      <c r="R9" s="36">
-        <f t="shared" si="2"/>
+      <c r="R9" s="31">
+        <f t="shared" si="5"/>
         <v>0.76</v>
       </c>
-      <c r="S9" s="36">
-        <f t="shared" si="3"/>
-        <v>0.612973308504036</v>
-      </c>
-      <c r="T9" s="36">
-        <f t="shared" si="4"/>
+      <c r="S9" s="31">
+        <f t="shared" si="6"/>
+        <v>0.612973308504035</v>
+      </c>
+      <c r="T9" s="31">
+        <f t="shared" si="7"/>
         <v>0.980679546968688</v>
       </c>
-      <c r="U9" s="36">
-        <f t="shared" si="5"/>
+      <c r="U9" s="31">
+        <f t="shared" si="8"/>
         <v>0.456859093730603</v>
       </c>
-      <c r="V9" s="37">
-        <f t="shared" si="6"/>
-        <v>0.795442501324854</v>
+      <c r="V9" s="32">
+        <f t="shared" si="9"/>
+        <v>0.665513877804381</v>
       </c>
     </row>
     <row r="10" s="4" customFormat="1" spans="1:22">
-      <c r="A10" s="11">
+      <c r="A10" s="21">
         <v>46078</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="E10" s="12">
-        <f t="shared" ref="E10:E19" si="7">F9</f>
+        <v>59</v>
+      </c>
+      <c r="E10" s="22">
+        <f t="shared" ref="E10:E19" si="10">F9</f>
         <v>0.375</v>
       </c>
-      <c r="F10" s="12">
+      <c r="F10" s="22">
         <v>0.416666666666667</v>
       </c>
-      <c r="G10" s="13">
-        <v>1829</v>
-      </c>
-      <c r="H10" s="13">
+      <c r="G10" s="23">
+        <f t="shared" si="0"/>
+        <v>2181.2</v>
+      </c>
+      <c r="H10" s="23">
         <v>1757</v>
       </c>
-      <c r="I10" s="13">
+      <c r="I10" s="23">
         <v>91</v>
       </c>
-      <c r="J10" s="22">
+      <c r="J10" s="24">
         <v>1666</v>
       </c>
-      <c r="K10" s="23">
+      <c r="K10" s="25">
         <v>1</v>
       </c>
-      <c r="L10" s="24">
+      <c r="L10" s="26">
         <v>0.3</v>
       </c>
-      <c r="M10" s="25">
-        <f t="shared" si="0"/>
+      <c r="M10" s="27">
+        <f t="shared" si="1"/>
         <v>0.7</v>
       </c>
-      <c r="N10" s="26">
+      <c r="N10" s="28">
         <v>0.000320924261874198</v>
       </c>
-      <c r="O10" s="14">
-        <f t="shared" si="1"/>
+      <c r="O10" s="29">
+        <f t="shared" si="2"/>
         <v>3116</v>
       </c>
-      <c r="P10" s="27">
-        <f>IF(M10=0," ",IFERROR(IF($P$1=1,H10/O10,H10*N10)," "))</f>
+      <c r="P10" s="30">
+        <f t="shared" si="3"/>
         <v>0.563863928112966</v>
       </c>
-      <c r="Q10" s="27">
-        <f>IFERROR(IF($Q$1=1,J10/O10,J10*N10)," ")</f>
+      <c r="Q10" s="30">
+        <f t="shared" si="4"/>
         <v>0.534659820282414</v>
       </c>
-      <c r="R10" s="36">
-        <f t="shared" si="2"/>
+      <c r="R10" s="31">
+        <f t="shared" si="5"/>
         <v>0.7</v>
       </c>
-      <c r="S10" s="36">
-        <f t="shared" si="3"/>
+      <c r="S10" s="31">
+        <f t="shared" si="6"/>
         <v>0.805519897304237</v>
       </c>
-      <c r="T10" s="36">
-        <f t="shared" si="4"/>
+      <c r="T10" s="31">
+        <f t="shared" si="7"/>
         <v>0.948207171314741</v>
       </c>
-      <c r="U10" s="36">
-        <f t="shared" si="5"/>
+      <c r="U10" s="31">
+        <f t="shared" si="8"/>
         <v>0.534659820282414</v>
       </c>
-      <c r="V10" s="37">
-        <f t="shared" si="6"/>
-        <v>0.960634226353199</v>
+      <c r="V10" s="32">
+        <f t="shared" si="9"/>
+        <v>0.805519897304236</v>
       </c>
     </row>
     <row r="11" s="4" customFormat="1" spans="1:22">
-      <c r="A11" s="11">
+      <c r="A11" s="21">
         <v>46078</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="E11" s="12">
+        <v>59</v>
+      </c>
+      <c r="E11" s="22">
+        <f t="shared" si="10"/>
+        <v>0.416666666666667</v>
+      </c>
+      <c r="F11" s="22">
+        <v>0.458333333333333</v>
+      </c>
+      <c r="G11" s="23">
+        <f t="shared" si="0"/>
+        <v>2770.6</v>
+      </c>
+      <c r="H11" s="23">
+        <v>1825</v>
+      </c>
+      <c r="I11" s="23">
+        <v>73</v>
+      </c>
+      <c r="J11" s="24">
+        <v>1752</v>
+      </c>
+      <c r="K11" s="25">
+        <v>1</v>
+      </c>
+      <c r="L11" s="26">
+        <v>0.5</v>
+      </c>
+      <c r="M11" s="27">
+        <f t="shared" si="1"/>
+        <v>0.5</v>
+      </c>
+      <c r="N11" s="28">
+        <v>0.000252652854977261</v>
+      </c>
+      <c r="O11" s="29">
+        <f t="shared" si="2"/>
+        <v>3958</v>
+      </c>
+      <c r="P11" s="30">
+        <f t="shared" si="3"/>
+        <v>0.461091460333501</v>
+      </c>
+      <c r="Q11" s="30">
+        <f t="shared" si="4"/>
+        <v>0.442647801920161</v>
+      </c>
+      <c r="R11" s="31">
+        <f t="shared" si="5"/>
+        <v>0.5</v>
+      </c>
+      <c r="S11" s="31">
+        <f t="shared" si="6"/>
+        <v>0.922182920667003</v>
+      </c>
+      <c r="T11" s="31">
         <f t="shared" si="7"/>
-        <v>0.416666666666667</v>
-      </c>
-      <c r="F11" s="12">
-        <v>0.458333333333333</v>
-      </c>
-      <c r="G11" s="13">
-        <v>1921</v>
-      </c>
-      <c r="H11" s="13">
-        <v>1825</v>
-      </c>
-      <c r="I11" s="13">
-        <v>73</v>
-      </c>
-      <c r="J11" s="22">
-        <v>1752</v>
-      </c>
-      <c r="K11" s="23">
-        <v>1</v>
-      </c>
-      <c r="L11" s="24">
-        <v>0.5</v>
-      </c>
-      <c r="M11" s="25">
-        <f t="shared" si="0"/>
-        <v>0.5</v>
-      </c>
-      <c r="N11" s="26">
-        <v>0.000252652854977261</v>
-      </c>
-      <c r="O11" s="14">
-        <f t="shared" si="1"/>
-        <v>3958</v>
-      </c>
-      <c r="P11" s="27">
-        <f>IF(M11=0," ",IFERROR(IF($P$1=1,H11/O11,H11*N11)," "))</f>
-        <v>0.461091460333501</v>
-      </c>
-      <c r="Q11" s="27">
-        <f>IFERROR(IF($Q$1=1,J11/O11,J11*N11)," ")</f>
+        <v>0.96</v>
+      </c>
+      <c r="U11" s="31">
+        <f t="shared" si="8"/>
         <v>0.442647801920161</v>
       </c>
-      <c r="R11" s="36">
-        <f t="shared" si="2"/>
-        <v>0.5</v>
-      </c>
-      <c r="S11" s="36">
-        <f t="shared" si="3"/>
-        <v>0.922182920667002</v>
-      </c>
-      <c r="T11" s="36">
-        <f t="shared" si="4"/>
-        <v>0.96</v>
-      </c>
-      <c r="U11" s="36">
-        <f t="shared" si="5"/>
-        <v>0.442647801920161</v>
-      </c>
-      <c r="V11" s="37">
-        <f t="shared" si="6"/>
-        <v>0.950026028110359</v>
+      <c r="V11" s="32">
+        <f t="shared" si="9"/>
+        <v>0.658702086190717</v>
       </c>
     </row>
     <row r="12" s="4" customFormat="1" spans="1:22">
-      <c r="A12" s="11">
+      <c r="A12" s="21">
         <v>46078</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="E12" s="12">
+        <v>59</v>
+      </c>
+      <c r="E12" s="22">
+        <f t="shared" si="10"/>
+        <v>0.458333333333333</v>
+      </c>
+      <c r="F12" s="22">
+        <v>0.5</v>
+      </c>
+      <c r="G12" s="23">
+        <f t="shared" si="0"/>
+        <v>2401.7</v>
+      </c>
+      <c r="H12" s="23">
+        <v>1642</v>
+      </c>
+      <c r="I12" s="23">
+        <v>77</v>
+      </c>
+      <c r="J12" s="24">
+        <v>1565</v>
+      </c>
+      <c r="K12" s="25">
+        <v>1</v>
+      </c>
+      <c r="L12" s="26">
+        <v>0.4</v>
+      </c>
+      <c r="M12" s="27">
+        <f t="shared" si="1"/>
+        <v>0.6</v>
+      </c>
+      <c r="N12" s="28">
+        <v>0.00029146021568056</v>
+      </c>
+      <c r="O12" s="29">
+        <f t="shared" si="2"/>
+        <v>3431</v>
+      </c>
+      <c r="P12" s="30">
+        <f t="shared" si="3"/>
+        <v>0.47857767414748</v>
+      </c>
+      <c r="Q12" s="30">
+        <f t="shared" si="4"/>
+        <v>0.456135237540076</v>
+      </c>
+      <c r="R12" s="31">
+        <f t="shared" si="5"/>
+        <v>0.6</v>
+      </c>
+      <c r="S12" s="31">
+        <f t="shared" si="6"/>
+        <v>0.797629456912466</v>
+      </c>
+      <c r="T12" s="31">
         <f t="shared" si="7"/>
-        <v>0.458333333333333</v>
-      </c>
-      <c r="F12" s="12">
-        <v>0.5</v>
-      </c>
-      <c r="G12" s="13">
-        <v>1820</v>
-      </c>
-      <c r="H12" s="13">
-        <v>1642</v>
-      </c>
-      <c r="I12" s="13">
-        <v>77</v>
-      </c>
-      <c r="J12" s="22">
-        <v>1565</v>
-      </c>
-      <c r="K12" s="23">
-        <v>1</v>
-      </c>
-      <c r="L12" s="24">
-        <v>0.4</v>
-      </c>
-      <c r="M12" s="25">
-        <f t="shared" si="0"/>
-        <v>0.6</v>
-      </c>
-      <c r="N12" s="26">
-        <v>0.00029146021568056</v>
-      </c>
-      <c r="O12" s="14">
-        <f t="shared" si="1"/>
-        <v>3431</v>
-      </c>
-      <c r="P12" s="27">
-        <f>IF(M12=0," ",IFERROR(IF($P$1=1,H12/O12,H12*N12)," "))</f>
-        <v>0.47857767414748</v>
-      </c>
-      <c r="Q12" s="27">
-        <f>IFERROR(IF($Q$1=1,J12/O12,J12*N12)," ")</f>
+        <v>0.953105968331302</v>
+      </c>
+      <c r="U12" s="31">
+        <f t="shared" si="8"/>
         <v>0.456135237540076</v>
       </c>
-      <c r="R12" s="36">
-        <f t="shared" si="2"/>
-        <v>0.6</v>
-      </c>
-      <c r="S12" s="36">
-        <f t="shared" si="3"/>
-        <v>0.797629456912467</v>
-      </c>
-      <c r="T12" s="36">
-        <f t="shared" si="4"/>
-        <v>0.953105968331302</v>
-      </c>
-      <c r="U12" s="36">
-        <f t="shared" si="5"/>
-        <v>0.456135237540076</v>
-      </c>
-      <c r="V12" s="37">
-        <f t="shared" si="6"/>
-        <v>0.902197802197802</v>
+      <c r="V12" s="32">
+        <f t="shared" si="9"/>
+        <v>0.683682391639256</v>
       </c>
     </row>
     <row r="13" s="4" customFormat="1" spans="1:22">
-      <c r="A13" s="11">
+      <c r="A13" s="21">
         <v>46078</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="E13" s="12">
+        <v>59</v>
+      </c>
+      <c r="E13" s="22">
+        <f t="shared" si="10"/>
+        <v>0.5</v>
+      </c>
+      <c r="F13" s="22">
+        <v>0.541666666666667</v>
+      </c>
+      <c r="G13" s="23">
+        <f t="shared" si="0"/>
+        <v>2480.1</v>
+      </c>
+      <c r="H13" s="23">
+        <v>1596</v>
+      </c>
+      <c r="I13" s="23">
+        <v>12</v>
+      </c>
+      <c r="J13" s="24">
+        <v>1584</v>
+      </c>
+      <c r="K13" s="25">
+        <v>1</v>
+      </c>
+      <c r="L13" s="26">
+        <v>0.2</v>
+      </c>
+      <c r="M13" s="27">
+        <f t="shared" si="1"/>
+        <v>0.8</v>
+      </c>
+      <c r="N13" s="28">
+        <v>0.000282246683601468</v>
+      </c>
+      <c r="O13" s="29">
+        <f t="shared" si="2"/>
+        <v>3543</v>
+      </c>
+      <c r="P13" s="30">
+        <f t="shared" si="3"/>
+        <v>0.450465707027943</v>
+      </c>
+      <c r="Q13" s="30">
+        <f t="shared" si="4"/>
+        <v>0.447078746824725</v>
+      </c>
+      <c r="R13" s="31">
+        <f t="shared" si="5"/>
+        <v>0.8</v>
+      </c>
+      <c r="S13" s="31">
+        <f t="shared" si="6"/>
+        <v>0.563082133784929</v>
+      </c>
+      <c r="T13" s="31">
         <f t="shared" si="7"/>
-        <v>0.5</v>
-      </c>
-      <c r="F13" s="12">
-        <v>0.541666666666667</v>
-      </c>
-      <c r="G13" s="13">
-        <v>1907</v>
-      </c>
-      <c r="H13" s="13">
-        <v>1596</v>
-      </c>
-      <c r="I13" s="13">
-        <v>12</v>
-      </c>
-      <c r="J13" s="22">
-        <v>1584</v>
-      </c>
-      <c r="K13" s="23">
-        <v>1</v>
-      </c>
-      <c r="L13" s="24">
-        <v>0.2</v>
-      </c>
-      <c r="M13" s="25">
-        <f t="shared" si="0"/>
-        <v>0.8</v>
-      </c>
-      <c r="N13" s="26">
-        <v>0.000282246683601468</v>
-      </c>
-      <c r="O13" s="14">
-        <f t="shared" si="1"/>
-        <v>3543</v>
-      </c>
-      <c r="P13" s="27">
-        <f>IF(M13=0," ",IFERROR(IF($P$1=1,H13/O13,H13*N13)," "))</f>
-        <v>0.450465707027943</v>
-      </c>
-      <c r="Q13" s="27">
-        <f>IFERROR(IF($Q$1=1,J13/O13,J13*N13)," ")</f>
+        <v>0.992481203007518</v>
+      </c>
+      <c r="U13" s="31">
+        <f t="shared" si="8"/>
         <v>0.447078746824725</v>
       </c>
-      <c r="R13" s="36">
-        <f t="shared" si="2"/>
-        <v>0.8</v>
-      </c>
-      <c r="S13" s="36">
-        <f t="shared" si="3"/>
-        <v>0.563082133784929</v>
-      </c>
-      <c r="T13" s="36">
-        <f t="shared" si="4"/>
-        <v>0.992481203007518</v>
-      </c>
-      <c r="U13" s="36">
-        <f t="shared" si="5"/>
-        <v>0.447078746824725</v>
-      </c>
-      <c r="V13" s="37">
-        <f t="shared" si="6"/>
-        <v>0.836916622968013</v>
+      <c r="V13" s="32">
+        <f t="shared" si="9"/>
+        <v>0.643522438611346</v>
       </c>
     </row>
     <row r="14" s="4" customFormat="1" spans="1:22">
-      <c r="A14" s="11">
+      <c r="A14" s="21">
         <v>46078</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="E14" s="12">
+        <v>59</v>
+      </c>
+      <c r="E14" s="22">
+        <f t="shared" si="10"/>
+        <v>0.541666666666667</v>
+      </c>
+      <c r="F14" s="22">
+        <v>0.583333333333333</v>
+      </c>
+      <c r="G14" s="23">
+        <f t="shared" si="0"/>
+        <v>2201.5</v>
+      </c>
+      <c r="H14" s="23">
+        <v>1890</v>
+      </c>
+      <c r="I14" s="23">
+        <v>34</v>
+      </c>
+      <c r="J14" s="24">
+        <v>1856</v>
+      </c>
+      <c r="K14" s="25">
+        <v>1</v>
+      </c>
+      <c r="L14" s="26">
+        <v>0.3</v>
+      </c>
+      <c r="M14" s="27">
+        <f t="shared" si="1"/>
+        <v>0.7</v>
+      </c>
+      <c r="N14" s="28">
+        <v>0.000317965023847377</v>
+      </c>
+      <c r="O14" s="29">
+        <f t="shared" si="2"/>
+        <v>3145</v>
+      </c>
+      <c r="P14" s="30">
+        <f t="shared" si="3"/>
+        <v>0.600953895071543</v>
+      </c>
+      <c r="Q14" s="30">
+        <f t="shared" si="4"/>
+        <v>0.590143084260732</v>
+      </c>
+      <c r="R14" s="31">
+        <f t="shared" si="5"/>
+        <v>0.7</v>
+      </c>
+      <c r="S14" s="31">
+        <f t="shared" si="6"/>
+        <v>0.858505564387918</v>
+      </c>
+      <c r="T14" s="31">
         <f t="shared" si="7"/>
-        <v>0.541666666666667</v>
-      </c>
-      <c r="F14" s="12">
-        <v>0.583333333333333</v>
-      </c>
-      <c r="G14" s="13">
-        <v>1916</v>
-      </c>
-      <c r="H14" s="13">
-        <v>1890</v>
-      </c>
-      <c r="I14" s="13">
-        <v>34</v>
-      </c>
-      <c r="J14" s="22">
-        <v>1856</v>
-      </c>
-      <c r="K14" s="23">
-        <v>1</v>
-      </c>
-      <c r="L14" s="24">
-        <v>0.3</v>
-      </c>
-      <c r="M14" s="25">
-        <f t="shared" si="0"/>
-        <v>0.7</v>
-      </c>
-      <c r="N14" s="26">
-        <v>0.000317965023847377</v>
-      </c>
-      <c r="O14" s="14">
-        <f t="shared" si="1"/>
-        <v>3145</v>
-      </c>
-      <c r="P14" s="27">
-        <f>IF(M14=0," ",IFERROR(IF($P$1=1,H14/O14,H14*N14)," "))</f>
-        <v>0.600953895071543</v>
-      </c>
-      <c r="Q14" s="27">
-        <f>IFERROR(IF($Q$1=1,J14/O14,J14*N14)," ")</f>
+        <v>0.982010582010583</v>
+      </c>
+      <c r="U14" s="31">
+        <f t="shared" si="8"/>
         <v>0.590143084260732</v>
       </c>
-      <c r="R14" s="36">
-        <f t="shared" si="2"/>
-        <v>0.7</v>
-      </c>
-      <c r="S14" s="36">
-        <f t="shared" si="3"/>
-        <v>0.858505564387919</v>
-      </c>
-      <c r="T14" s="36">
-        <f t="shared" si="4"/>
-        <v>0.982010582010582</v>
-      </c>
-      <c r="U14" s="36">
-        <f t="shared" si="5"/>
-        <v>0.590143084260732</v>
-      </c>
-      <c r="V14" s="37">
-        <f t="shared" si="6"/>
-        <v>0.98643006263048</v>
+      <c r="V14" s="32">
+        <f t="shared" si="9"/>
+        <v>0.858505564387917</v>
       </c>
     </row>
     <row r="15" s="4" customFormat="1" spans="1:22">
-      <c r="A15" s="11">
+      <c r="A15" s="21">
         <v>46078</v>
       </c>
       <c r="B15" s="4" t="str">
@@ -2911,78 +2960,79 @@
         <v>NKD</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="E15" s="12">
+        <v>69</v>
+      </c>
+      <c r="E15" s="22">
+        <f t="shared" si="10"/>
+        <v>0.583333333333333</v>
+      </c>
+      <c r="F15" s="22">
+        <v>0.625</v>
+      </c>
+      <c r="G15" s="23">
+        <f>$G$2*O15*K15</f>
+        <v>2369.5</v>
+      </c>
+      <c r="H15" s="23">
+        <v>1678</v>
+      </c>
+      <c r="I15" s="23">
+        <v>57</v>
+      </c>
+      <c r="J15" s="24">
+        <v>1621</v>
+      </c>
+      <c r="K15" s="25">
+        <v>1</v>
+      </c>
+      <c r="L15" s="26">
+        <v>0.15</v>
+      </c>
+      <c r="M15" s="27">
+        <f t="shared" si="1"/>
+        <v>0.85</v>
+      </c>
+      <c r="N15" s="28">
+        <v>0.000295420974889217</v>
+      </c>
+      <c r="O15" s="29">
+        <f t="shared" si="2"/>
+        <v>3385</v>
+      </c>
+      <c r="P15" s="30">
+        <f t="shared" si="3"/>
+        <v>0.495716395864106</v>
+      </c>
+      <c r="Q15" s="30">
+        <f t="shared" si="4"/>
+        <v>0.478877400295421</v>
+      </c>
+      <c r="R15" s="31">
+        <f t="shared" si="5"/>
+        <v>0.85</v>
+      </c>
+      <c r="S15" s="31">
+        <f t="shared" si="6"/>
+        <v>0.583195759840125</v>
+      </c>
+      <c r="T15" s="31">
         <f t="shared" si="7"/>
-        <v>0.583333333333333</v>
-      </c>
-      <c r="F15" s="12">
-        <v>0.625</v>
-      </c>
-      <c r="G15" s="13">
-        <v>1865</v>
-      </c>
-      <c r="H15" s="13">
-        <v>1678</v>
-      </c>
-      <c r="I15" s="13">
-        <v>57</v>
-      </c>
-      <c r="J15" s="22">
-        <v>1621</v>
-      </c>
-      <c r="K15" s="23">
-        <v>1</v>
-      </c>
-      <c r="L15" s="24">
-        <v>0.15</v>
-      </c>
-      <c r="M15" s="25">
-        <f t="shared" si="0"/>
-        <v>0.85</v>
-      </c>
-      <c r="N15" s="26">
-        <v>0.000295420974889217</v>
-      </c>
-      <c r="O15" s="14">
-        <f t="shared" si="1"/>
-        <v>3385</v>
-      </c>
-      <c r="P15" s="27">
-        <f>IF(M15=0," ",IFERROR(IF($P$1=1,H15/O15,H15*N15)," "))</f>
-        <v>0.495716395864106</v>
-      </c>
-      <c r="Q15" s="27">
-        <f>IFERROR(IF($Q$1=1,J15/O15,J15*N15)," ")</f>
+        <v>0.966030989272944</v>
+      </c>
+      <c r="U15" s="31">
+        <f t="shared" si="8"/>
         <v>0.478877400295421</v>
       </c>
-      <c r="R15" s="36">
-        <f t="shared" si="2"/>
-        <v>0.85</v>
-      </c>
-      <c r="S15" s="36">
-        <f t="shared" si="3"/>
-        <v>0.583195759840125</v>
-      </c>
-      <c r="T15" s="36">
-        <f t="shared" si="4"/>
-        <v>0.966030989272945</v>
-      </c>
-      <c r="U15" s="36">
-        <f t="shared" si="5"/>
-        <v>0.478877400295421</v>
-      </c>
-      <c r="V15" s="37">
-        <f t="shared" si="6"/>
-        <v>0.899731903485255</v>
+      <c r="V15" s="32">
+        <f t="shared" si="9"/>
+        <v>0.708166279805866</v>
       </c>
     </row>
     <row r="16" s="4" customFormat="1" spans="1:22">
-      <c r="A16" s="11">
+      <c r="A16" s="21">
         <v>46078</v>
       </c>
       <c r="B16" s="4" t="str">
@@ -2990,78 +3040,79 @@
         <v>CR4</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D16" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="E16" s="22">
+        <f t="shared" si="10"/>
+        <v>0.625</v>
+      </c>
+      <c r="F16" s="22">
+        <v>0.666666666666667</v>
+      </c>
+      <c r="G16" s="23">
+        <f>$G$2*O16*K16</f>
+        <v>2149</v>
+      </c>
+      <c r="H16" s="23">
+        <v>1745</v>
+      </c>
+      <c r="I16" s="23">
         <v>67</v>
       </c>
-      <c r="E16" s="12">
+      <c r="J16" s="24">
+        <v>1678</v>
+      </c>
+      <c r="K16" s="25">
+        <v>1</v>
+      </c>
+      <c r="L16" s="26">
+        <v>0.25</v>
+      </c>
+      <c r="M16" s="27">
+        <f t="shared" si="1"/>
+        <v>0.75</v>
+      </c>
+      <c r="N16" s="28">
+        <v>0.000325732899022801</v>
+      </c>
+      <c r="O16" s="29">
+        <f t="shared" si="2"/>
+        <v>3070</v>
+      </c>
+      <c r="P16" s="30">
+        <f t="shared" si="3"/>
+        <v>0.568403908794788</v>
+      </c>
+      <c r="Q16" s="30">
+        <f t="shared" si="4"/>
+        <v>0.54657980456026</v>
+      </c>
+      <c r="R16" s="31">
+        <f t="shared" si="5"/>
+        <v>0.75</v>
+      </c>
+      <c r="S16" s="31">
+        <f t="shared" si="6"/>
+        <v>0.75787187839305</v>
+      </c>
+      <c r="T16" s="31">
         <f t="shared" si="7"/>
-        <v>0.625</v>
-      </c>
-      <c r="F16" s="12">
-        <v>0.666666666666667</v>
-      </c>
-      <c r="G16" s="13">
-        <v>1938.88888888889</v>
-      </c>
-      <c r="H16" s="13">
-        <v>1745</v>
-      </c>
-      <c r="I16" s="13">
-        <v>67</v>
-      </c>
-      <c r="J16" s="22">
-        <v>1678</v>
-      </c>
-      <c r="K16" s="23">
-        <v>1</v>
-      </c>
-      <c r="L16" s="24">
-        <v>0.25</v>
-      </c>
-      <c r="M16" s="25">
-        <f t="shared" si="0"/>
-        <v>0.75</v>
-      </c>
-      <c r="N16" s="26">
-        <v>0.000325732899022801</v>
-      </c>
-      <c r="O16" s="14">
-        <f t="shared" si="1"/>
-        <v>3070</v>
-      </c>
-      <c r="P16" s="27">
-        <f>IF(M16=0," ",IFERROR(IF($P$1=1,H16/O16,H16*N16)," "))</f>
-        <v>0.568403908794788</v>
-      </c>
-      <c r="Q16" s="27">
-        <f>IFERROR(IF($Q$1=1,J16/O16,J16*N16)," ")</f>
+        <v>0.961604584527221</v>
+      </c>
+      <c r="U16" s="31">
+        <f t="shared" si="8"/>
         <v>0.54657980456026</v>
       </c>
-      <c r="R16" s="36">
-        <f t="shared" si="2"/>
-        <v>0.75</v>
-      </c>
-      <c r="S16" s="36">
-        <f t="shared" si="3"/>
-        <v>0.757871878393051</v>
-      </c>
-      <c r="T16" s="36">
-        <f t="shared" si="4"/>
-        <v>0.96160458452722</v>
-      </c>
-      <c r="U16" s="36">
-        <f t="shared" si="5"/>
-        <v>0.54657980456026</v>
-      </c>
-      <c r="V16" s="37">
-        <f t="shared" si="6"/>
-        <v>0.899999999999999</v>
+      <c r="V16" s="32">
+        <f t="shared" si="9"/>
+        <v>0.812005583992555</v>
       </c>
     </row>
     <row r="17" s="4" customFormat="1" spans="1:22">
-      <c r="A17" s="11">
+      <c r="A17" s="21">
         <v>46078</v>
       </c>
       <c r="B17" s="4" t="str">
@@ -3069,78 +3120,79 @@
         <v>DSS</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="E17" s="12">
+        <v>69</v>
+      </c>
+      <c r="E17" s="22">
+        <f t="shared" si="10"/>
+        <v>0.666666666666667</v>
+      </c>
+      <c r="F17" s="22">
+        <v>0.708333333333333</v>
+      </c>
+      <c r="G17" s="23">
+        <f>$G$2*O17*K17</f>
+        <v>2255.4</v>
+      </c>
+      <c r="H17" s="23">
+        <v>1509</v>
+      </c>
+      <c r="I17" s="23">
+        <v>54</v>
+      </c>
+      <c r="J17" s="24">
+        <v>1455</v>
+      </c>
+      <c r="K17" s="25">
+        <v>1</v>
+      </c>
+      <c r="L17" s="26">
+        <v>0.22</v>
+      </c>
+      <c r="M17" s="27">
+        <f t="shared" si="1"/>
+        <v>0.78</v>
+      </c>
+      <c r="N17" s="28">
+        <v>0.000310366232153942</v>
+      </c>
+      <c r="O17" s="29">
+        <f t="shared" si="2"/>
+        <v>3222</v>
+      </c>
+      <c r="P17" s="30">
+        <f t="shared" si="3"/>
+        <v>0.468342644320298</v>
+      </c>
+      <c r="Q17" s="30">
+        <f t="shared" si="4"/>
+        <v>0.451582867783986</v>
+      </c>
+      <c r="R17" s="31">
+        <f t="shared" si="5"/>
+        <v>0.78</v>
+      </c>
+      <c r="S17" s="31">
+        <f t="shared" si="6"/>
+        <v>0.600439287590126</v>
+      </c>
+      <c r="T17" s="31">
         <f t="shared" si="7"/>
-        <v>0.666666666666667</v>
-      </c>
-      <c r="F17" s="12">
-        <v>0.708333333333333</v>
-      </c>
-      <c r="G17" s="13">
-        <v>1676.66666666667</v>
-      </c>
-      <c r="H17" s="13">
-        <v>1509</v>
-      </c>
-      <c r="I17" s="13">
-        <v>54</v>
-      </c>
-      <c r="J17" s="22">
-        <v>1455</v>
-      </c>
-      <c r="K17" s="23">
-        <v>1</v>
-      </c>
-      <c r="L17" s="24">
-        <v>0.22</v>
-      </c>
-      <c r="M17" s="25">
-        <f t="shared" si="0"/>
-        <v>0.78</v>
-      </c>
-      <c r="N17" s="26">
-        <v>0.000310366232153942</v>
-      </c>
-      <c r="O17" s="14">
-        <f t="shared" si="1"/>
-        <v>3222</v>
-      </c>
-      <c r="P17" s="27">
-        <f>IF(M17=0," ",IFERROR(IF($P$1=1,H17/O17,H17*N17)," "))</f>
-        <v>0.468342644320298</v>
-      </c>
-      <c r="Q17" s="27">
-        <f>IFERROR(IF($Q$1=1,J17/O17,J17*N17)," ")</f>
+        <v>0.964214711729623</v>
+      </c>
+      <c r="U17" s="31">
+        <f t="shared" si="8"/>
         <v>0.451582867783986</v>
       </c>
-      <c r="R17" s="36">
-        <f t="shared" si="2"/>
-        <v>0.78</v>
-      </c>
-      <c r="S17" s="36">
-        <f t="shared" si="3"/>
-        <v>0.600439287590126</v>
-      </c>
-      <c r="T17" s="36">
-        <f t="shared" si="4"/>
-        <v>0.964214711729624</v>
-      </c>
-      <c r="U17" s="36">
-        <f t="shared" si="5"/>
-        <v>0.451582867783986</v>
-      </c>
-      <c r="V17" s="37">
-        <f t="shared" si="6"/>
-        <v>0.899999999999998</v>
+      <c r="V17" s="32">
+        <f t="shared" si="9"/>
+        <v>0.669060920457569</v>
       </c>
     </row>
     <row r="18" s="4" customFormat="1" spans="1:22">
-      <c r="A18" s="11">
+      <c r="A18" s="21">
         <v>46078</v>
       </c>
       <c r="B18" s="4" t="str">
@@ -3148,78 +3200,79 @@
         <v>SP</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="E18" s="12">
+        <v>69</v>
+      </c>
+      <c r="E18" s="22">
+        <f t="shared" si="10"/>
+        <v>0.708333333333333</v>
+      </c>
+      <c r="F18" s="22">
+        <v>0.75</v>
+      </c>
+      <c r="G18" s="23">
+        <f>$G$2*O18*K18</f>
+        <v>2181.2</v>
+      </c>
+      <c r="H18" s="23">
+        <v>1518</v>
+      </c>
+      <c r="I18" s="23">
+        <v>27</v>
+      </c>
+      <c r="J18" s="24">
+        <v>1491</v>
+      </c>
+      <c r="K18" s="25">
+        <v>1</v>
+      </c>
+      <c r="L18" s="26">
+        <v>0.27</v>
+      </c>
+      <c r="M18" s="27">
+        <f t="shared" si="1"/>
+        <v>0.73</v>
+      </c>
+      <c r="N18" s="28">
+        <v>0.000320924261874198</v>
+      </c>
+      <c r="O18" s="29">
+        <f t="shared" si="2"/>
+        <v>3116</v>
+      </c>
+      <c r="P18" s="30">
+        <f t="shared" si="3"/>
+        <v>0.487163029525033</v>
+      </c>
+      <c r="Q18" s="30">
+        <f t="shared" si="4"/>
+        <v>0.478498074454429</v>
+      </c>
+      <c r="R18" s="31">
+        <f t="shared" si="5"/>
+        <v>0.73</v>
+      </c>
+      <c r="S18" s="31">
+        <f t="shared" si="6"/>
+        <v>0.667346615787716</v>
+      </c>
+      <c r="T18" s="31">
         <f t="shared" si="7"/>
-        <v>0.708333333333333</v>
-      </c>
-      <c r="F18" s="12">
-        <v>0.75</v>
-      </c>
-      <c r="G18" s="13">
-        <v>1686.66666666667</v>
-      </c>
-      <c r="H18" s="13">
-        <v>1518</v>
-      </c>
-      <c r="I18" s="13">
-        <v>27</v>
-      </c>
-      <c r="J18" s="22">
-        <v>1491</v>
-      </c>
-      <c r="K18" s="23">
-        <v>1</v>
-      </c>
-      <c r="L18" s="24">
-        <v>0.27</v>
-      </c>
-      <c r="M18" s="25">
-        <f t="shared" si="0"/>
-        <v>0.73</v>
-      </c>
-      <c r="N18" s="26">
-        <v>0.000320924261874198</v>
-      </c>
-      <c r="O18" s="14">
-        <f t="shared" si="1"/>
-        <v>3116</v>
-      </c>
-      <c r="P18" s="27">
-        <f>IF(M18=0," ",IFERROR(IF($P$1=1,H18/O18,H18*N18)," "))</f>
-        <v>0.487163029525033</v>
-      </c>
-      <c r="Q18" s="27">
-        <f>IFERROR(IF($Q$1=1,J18/O18,J18*N18)," ")</f>
+        <v>0.982213438735177</v>
+      </c>
+      <c r="U18" s="31">
+        <f t="shared" si="8"/>
         <v>0.478498074454429</v>
       </c>
-      <c r="R18" s="36">
-        <f t="shared" si="2"/>
-        <v>0.73</v>
-      </c>
-      <c r="S18" s="36">
-        <f t="shared" si="3"/>
-        <v>0.667346615787716</v>
-      </c>
-      <c r="T18" s="36">
-        <f t="shared" si="4"/>
-        <v>0.982213438735177</v>
-      </c>
-      <c r="U18" s="36">
-        <f t="shared" si="5"/>
-        <v>0.478498074454429</v>
-      </c>
-      <c r="V18" s="37">
-        <f t="shared" si="6"/>
-        <v>0.899999999999998</v>
+      <c r="V18" s="32">
+        <f t="shared" si="9"/>
+        <v>0.69594718503576</v>
       </c>
     </row>
     <row r="19" s="4" customFormat="1" spans="1:22">
-      <c r="A19" s="11">
+      <c r="A19" s="21">
         <v>46078</v>
       </c>
       <c r="B19" s="4" t="str">
@@ -3227,175 +3280,176 @@
         <v>CHR</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="E19" s="12">
+        <v>69</v>
+      </c>
+      <c r="E19" s="22">
+        <f t="shared" si="10"/>
+        <v>0.75</v>
+      </c>
+      <c r="F19" s="22">
+        <v>0.791666666666667</v>
+      </c>
+      <c r="G19" s="23">
+        <f>$G$2*O19*K19</f>
+        <v>2770.6</v>
+      </c>
+      <c r="H19" s="23">
+        <v>1763</v>
+      </c>
+      <c r="I19" s="23">
+        <v>91</v>
+      </c>
+      <c r="J19" s="24">
+        <v>1672</v>
+      </c>
+      <c r="K19" s="25">
+        <v>1</v>
+      </c>
+      <c r="L19" s="26">
+        <v>0.4</v>
+      </c>
+      <c r="M19" s="27">
+        <f t="shared" si="1"/>
+        <v>0.6</v>
+      </c>
+      <c r="N19" s="28">
+        <v>0.000252652854977261</v>
+      </c>
+      <c r="O19" s="29">
+        <f t="shared" si="2"/>
+        <v>3958</v>
+      </c>
+      <c r="P19" s="30">
+        <f t="shared" si="3"/>
+        <v>0.445426983324911</v>
+      </c>
+      <c r="Q19" s="30">
+        <f t="shared" si="4"/>
+        <v>0.42243557352198</v>
+      </c>
+      <c r="R19" s="31">
+        <f t="shared" si="5"/>
+        <v>0.6</v>
+      </c>
+      <c r="S19" s="31">
+        <f t="shared" si="6"/>
+        <v>0.742378305541519</v>
+      </c>
+      <c r="T19" s="31">
         <f t="shared" si="7"/>
-        <v>0.75</v>
-      </c>
-      <c r="F19" s="12">
-        <v>0.791666666666667</v>
-      </c>
-      <c r="G19" s="13">
-        <v>1958.88888888889</v>
-      </c>
-      <c r="H19" s="13">
-        <v>1763</v>
-      </c>
-      <c r="I19" s="13">
-        <v>91</v>
-      </c>
-      <c r="J19" s="22">
-        <v>1672</v>
-      </c>
-      <c r="K19" s="23">
-        <v>1</v>
-      </c>
-      <c r="L19" s="24">
-        <v>0.4</v>
-      </c>
-      <c r="M19" s="25">
-        <f t="shared" si="0"/>
-        <v>0.6</v>
-      </c>
-      <c r="N19" s="26">
-        <v>0.000252652854977261</v>
-      </c>
-      <c r="O19" s="14">
-        <f t="shared" si="1"/>
-        <v>3958</v>
-      </c>
-      <c r="P19" s="27">
-        <f>IF(M19=0," ",IFERROR(IF($P$1=1,H19/O19,H19*N19)," "))</f>
-        <v>0.445426983324911</v>
-      </c>
-      <c r="Q19" s="27">
-        <f>IFERROR(IF($Q$1=1,J19/O19,J19*N19)," ")</f>
+        <v>0.948383437322744</v>
+      </c>
+      <c r="U19" s="31">
+        <f t="shared" si="8"/>
         <v>0.42243557352198</v>
       </c>
-      <c r="R19" s="36">
-        <f t="shared" si="2"/>
-        <v>0.6</v>
-      </c>
-      <c r="S19" s="36">
-        <f t="shared" si="3"/>
-        <v>0.742378305541518</v>
-      </c>
-      <c r="T19" s="36">
-        <f t="shared" si="4"/>
-        <v>0.948383437322745</v>
-      </c>
-      <c r="U19" s="36">
-        <f t="shared" si="5"/>
-        <v>0.42243557352198</v>
-      </c>
-      <c r="V19" s="37">
-        <f t="shared" si="6"/>
-        <v>0.899999999999999</v>
+      <c r="V19" s="32">
+        <f t="shared" si="9"/>
+        <v>0.636324261892731</v>
       </c>
     </row>
     <row r="20" s="4" customFormat="1" spans="1:22">
-      <c r="A20" s="11"/>
-      <c r="E20" s="12"/>
-      <c r="F20" s="12"/>
-      <c r="G20" s="14"/>
-      <c r="H20" s="14"/>
-      <c r="I20" s="14"/>
-      <c r="J20" s="14"/>
-      <c r="K20" s="28"/>
-      <c r="L20" s="29"/>
-      <c r="M20" s="29"/>
-      <c r="N20" s="30"/>
-      <c r="O20" s="14"/>
-      <c r="P20" s="30"/>
-      <c r="Q20" s="30"/>
-      <c r="R20" s="38"/>
-      <c r="S20" s="38"/>
-      <c r="T20" s="38"/>
-      <c r="U20" s="38"/>
-      <c r="V20" s="39"/>
+      <c r="A20" s="21"/>
+      <c r="E20" s="22"/>
+      <c r="F20" s="22"/>
+      <c r="G20" s="29"/>
+      <c r="H20" s="29"/>
+      <c r="I20" s="29"/>
+      <c r="J20" s="29"/>
+      <c r="K20" s="33"/>
+      <c r="L20" s="34"/>
+      <c r="M20" s="34"/>
+      <c r="N20" s="35"/>
+      <c r="O20" s="29"/>
+      <c r="P20" s="35"/>
+      <c r="Q20" s="35"/>
+      <c r="R20" s="36"/>
+      <c r="S20" s="36"/>
+      <c r="T20" s="36"/>
+      <c r="U20" s="36"/>
+      <c r="V20" s="37"/>
     </row>
     <row r="21" s="4" customFormat="1" ht="16.3" spans="1:22">
-      <c r="A21" s="11"/>
-      <c r="E21" s="12"/>
-      <c r="F21" s="12"/>
-      <c r="G21" s="15">
+      <c r="A21" s="21"/>
+      <c r="E21" s="22"/>
+      <c r="F21" s="22"/>
+      <c r="G21" s="38">
         <f>SUM(G7:G19)</f>
-        <v>24103.1111111111</v>
-      </c>
-      <c r="H21" s="15">
-        <f t="shared" ref="H21:N21" si="8">SUM(H7:H19)</f>
+        <v>30625</v>
+      </c>
+      <c r="H21" s="38">
+        <f t="shared" ref="H21:N21" si="11">SUM(H7:H19)</f>
         <v>21698</v>
       </c>
-      <c r="I21" s="15">
-        <f t="shared" si="8"/>
+      <c r="I21" s="38">
+        <f t="shared" si="11"/>
         <v>733</v>
       </c>
-      <c r="J21" s="15">
-        <f t="shared" si="8"/>
+      <c r="J21" s="38">
+        <f t="shared" si="11"/>
         <v>20965</v>
       </c>
-      <c r="K21" s="31">
-        <f t="shared" si="8"/>
+      <c r="K21" s="39">
+        <f t="shared" si="11"/>
         <v>13</v>
       </c>
-      <c r="L21" s="32">
-        <f t="shared" si="8"/>
+      <c r="L21" s="40">
+        <f t="shared" si="11"/>
         <v>3.73</v>
       </c>
-      <c r="M21" s="32">
-        <f t="shared" si="8"/>
+      <c r="M21" s="40">
+        <f t="shared" si="11"/>
         <v>9.27</v>
       </c>
-      <c r="N21" s="33">
-        <f t="shared" si="8"/>
+      <c r="N21" s="41">
+        <f t="shared" si="11"/>
         <v>0.00389102137586216</v>
       </c>
-      <c r="O21" s="15"/>
-      <c r="P21" s="33">
+      <c r="O21" s="38"/>
+      <c r="P21" s="41">
         <f>SUM(P7:P19)</f>
         <v>6.48008446263769</v>
       </c>
-      <c r="Q21" s="33">
+      <c r="Q21" s="41">
         <f>SUM(Q7:Q19)</f>
         <v>6.26293698874817</v>
       </c>
-      <c r="R21" s="40">
+      <c r="R21" s="42">
         <f>IFERROR(M21/K21," ")</f>
         <v>0.713076923076923</v>
       </c>
-      <c r="S21" s="40">
+      <c r="S21" s="42">
         <f>IFERROR(P21/M21," ")</f>
         <v>0.699038237609244</v>
       </c>
-      <c r="T21" s="40">
+      <c r="T21" s="42">
         <f>IFERROR(Q21/P21," ")</f>
-        <v>0.966490024143739</v>
-      </c>
-      <c r="U21" s="40">
+        <v>0.966490024143738</v>
+      </c>
+      <c r="U21" s="42">
         <f>IFERROR(Q21/K21," ")</f>
         <v>0.481764383749859</v>
       </c>
-      <c r="V21" s="41">
+      <c r="V21" s="43">
         <f>H21/G21</f>
-        <v>0.900215739784629</v>
+        <v>0.70850612244898</v>
       </c>
     </row>
-    <row r="22" spans="12:17">
-      <c r="L22" s="34"/>
-      <c r="Q22" s="42"/>
+    <row r="22" spans="1:22">
+      <c r="L22" s="44"/>
+      <c r="Q22" s="45"/>
     </row>
-    <row r="23" spans="12:12">
-      <c r="L23" s="34"/>
+    <row r="23" spans="1:22">
+      <c r="L23" s="44"/>
     </row>
-    <row r="24" spans="12:12">
-      <c r="L24" s="34"/>
+    <row r="24" spans="1:22">
+      <c r="L24" s="44"/>
     </row>
-    <row r="25" spans="12:12">
-      <c r="L25" s="34"/>
+    <row r="25" spans="1:22">
+      <c r="L25" s="44"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>